<commit_message>
Integrar cambios completos de Banco1 en proyecto Banco
</commit_message>
<xml_diff>
--- a/files/asientos.xlsx
+++ b/files/asientos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P805"/>
+  <dimension ref="A1:Q805"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -517,6 +517,11 @@
           <t>Correos</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1235,11 +1240,6 @@
       <c r="J18" t="n">
         <v>2401</v>
       </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>ENTIDAD PRESTADORA DE SERVICIOS DE SANEA</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1284,6 +1284,11 @@
           <t>UNIV NAC PEDRO RUIZ GALLO PTO 2003</t>
         </is>
       </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>minonanve@unprg.edu.pe</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1328,6 +1333,11 @@
           <t>UNIV NAC PEDRO RUIZ GALLO PTO 2003</t>
         </is>
       </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>minonanve@unprg.edu.pe</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1445,11 +1455,6 @@
       <c r="J23" t="n">
         <v>2401</v>
       </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>CONSORCIO ELECTRICO DE VILLACURI S.A.C.</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1641,11 +1646,6 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>WESTERN UNION PERU S.A.</t>
-        </is>
-      </c>
       <c r="O27" t="n">
         <v>7000002213</v>
       </c>
@@ -1830,6 +1830,11 @@
           <t>MUNI DIST MOCHUMI PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>u212prac01@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2006,6 +2011,11 @@
           <t>MUNI DIST ANGUIA</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>ronaldlabans@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2050,6 +2060,11 @@
           <t>REGION CAJAMARCA-CHOTA PPTO</t>
         </is>
       </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>carlosbva8@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2143,11 +2158,6 @@
       <c r="J38" t="n">
         <v>2401</v>
       </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
-        </is>
-      </c>
       <c r="O38" t="n">
         <v>7000002212</v>
       </c>
@@ -2479,6 +2489,11 @@
           <t>MUNI DIST LAJAS</t>
         </is>
       </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>tesoreria@munilajas.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2523,6 +2538,11 @@
           <t>MUNI DIST ANGUIA</t>
         </is>
       </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>ronaldlabans@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2567,6 +2587,11 @@
           <t>MUNI DIST ANGUIA</t>
         </is>
       </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>ronaldlabans@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2802,6 +2827,11 @@
           <t>DIREC AVIACION POLICIAL PTO 2003</t>
         </is>
       </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>depsam.lambayeque@policia.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2993,6 +3023,11 @@
           <t>SUPERINT NAC FISCALIZACION LABORAL-</t>
         </is>
       </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>lruizr@sunafil.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3140,11 +3175,6 @@
           <t>PAGO PROVEEDORES RIPLE</t>
         </is>
       </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>TIENDAS POR DEPARTAMENTO RIPLEY S.A.C.</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3189,6 +3219,11 @@
           <t>MUNI DIST ANGUIA</t>
         </is>
       </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>ronaldlabans@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3282,6 +3317,11 @@
           <t>ORG SUP INVERSION ENERGIA Y MINERIA</t>
         </is>
       </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>ycruzado@osinergmin.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4113,11 +4153,6 @@
           <t>Pago Fact.203712041620</t>
         </is>
       </c>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t>COMPANIA ELECTRICA EL PLATANAL S.A.</t>
-        </is>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4344,11 +4379,6 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t>WESTERN UNION PERU S.A.</t>
-        </is>
-      </c>
       <c r="O86" t="n">
         <v>7000002099</v>
       </c>
@@ -4729,11 +4759,6 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
-      <c r="L94" t="inlineStr">
-        <is>
-          <t>ON EMPRESAS S.A.C.</t>
-        </is>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4778,6 +4803,11 @@
           <t>IPD PPTO 2003</t>
         </is>
       </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>malvites@ipd.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4866,6 +4896,11 @@
           <t>MUNI DIST PITIPO PPTO</t>
         </is>
       </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>jvaleriano1112@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4996,6 +5031,11 @@
           <t>CENTRO DE FORMACION EN TURISMO</t>
         </is>
       </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>dllaguento@cenfotur.edu.pe</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5040,6 +5080,11 @@
           <t>REGION LAMBAYEQUE-AGRICULTURA PPTO</t>
         </is>
       </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>graservicios2024@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5204,11 +5249,6 @@
       <c r="J105" t="n">
         <v>2401</v>
       </c>
-      <c r="L105" t="inlineStr">
-        <is>
-          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
-        </is>
-      </c>
       <c r="O105" t="n">
         <v>7000002097</v>
       </c>
@@ -5599,6 +5639,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5752,11 +5797,6 @@
       <c r="J116" t="n">
         <v>2401</v>
       </c>
-      <c r="L116" t="inlineStr">
-        <is>
-          <t>ENTIDAD PRESTADORA DE SERVICIOS DE SANEA</t>
-        </is>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5845,6 +5885,11 @@
           <t>REGION LAMBAYEQUE-AGRICULTURA PPTO</t>
         </is>
       </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>graservicios2024@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -5889,6 +5934,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -6071,6 +6121,11 @@
           <t>MUNI DIST MIRACOSTA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>gorderiquev@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6115,6 +6170,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -6211,6 +6271,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6361,6 +6426,11 @@
           <t>MUNI DIST MIRACOSTA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>gorderiquev@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6452,6 +6522,11 @@
           <t>MUNI DIST MIRACOSTA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>gorderiquev@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6496,6 +6571,11 @@
           <t>MTC ADMINISTRACION GRAL PPTO 2003</t>
         </is>
       </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>apaicog@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6740,6 +6820,11 @@
           <t>MUNI DIST MIRACOSTA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>gorderiquev@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6784,6 +6869,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6828,6 +6918,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -6872,6 +6967,11 @@
           <t>GR CAJAMARCA-EDUCAC UGEL CELENDIN</t>
         </is>
       </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>abastecimientos@ugelcelendin.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6916,6 +7016,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -6960,6 +7065,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -7004,6 +7114,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -7048,6 +7163,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -7149,6 +7269,11 @@
           <t>MUNI DIST MIRACOSTA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>gorderiquev@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -7193,6 +7318,11 @@
           <t>MUNI DIST MIRACOSTA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>gorderiquev@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -7237,6 +7367,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -7281,6 +7416,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -8048,11 +8188,6 @@
       <c r="J167" t="n">
         <v>2401</v>
       </c>
-      <c r="L167" t="inlineStr">
-        <is>
-          <t>VIETTEL PERU S.A.C - CAJ</t>
-        </is>
-      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -8097,11 +8232,6 @@
           <t>Pago0002301550-2026-FE</t>
         </is>
       </c>
-      <c r="L168" t="inlineStr">
-        <is>
-          <t>FENIX POWER PERU S.A.</t>
-        </is>
-      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -8344,11 +8474,6 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
-      <c r="L173" t="inlineStr">
-        <is>
-          <t>WESTERN UNION PERU S.A.</t>
-        </is>
-      </c>
       <c r="O173" t="n">
         <v>7000002086</v>
       </c>
@@ -8526,6 +8651,11 @@
           <t>REGION CAJAMARCA-SALUD CUTERVO</t>
         </is>
       </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>fsoberon05@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -8760,11 +8890,6 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
-      <c r="L182" t="inlineStr">
-        <is>
-          <t>ALDEAS INFANTILES SOS PERU - ASOCIACION NACIONAL</t>
-        </is>
-      </c>
       <c r="O182" t="n">
         <v>7000002143</v>
       </c>
@@ -8807,11 +8932,6 @@
       <c r="J183" t="n">
         <v>2401</v>
       </c>
-      <c r="L183" t="inlineStr">
-        <is>
-          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
-        </is>
-      </c>
       <c r="O183" t="n">
         <v>7000002085</v>
       </c>
@@ -8854,11 +8974,6 @@
       <c r="J184" t="n">
         <v>2401</v>
       </c>
-      <c r="L184" t="inlineStr">
-        <is>
-          <t>REPRESENT.Y SERVICIOS - INGENIEROS SRL</t>
-        </is>
-      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -9299,11 +9414,6 @@
       <c r="J193" t="n">
         <v>2401</v>
       </c>
-      <c r="L193" t="inlineStr">
-        <is>
-          <t>REPRESENT.Y SERVICIOS - INGENIEROS SRL</t>
-        </is>
-      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -10931,11 +11041,6 @@
       <c r="J227" t="n">
         <v>2401</v>
       </c>
-      <c r="L227" t="inlineStr">
-        <is>
-          <t>EGEMSA</t>
-        </is>
-      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -11936,11 +12041,6 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
-      <c r="L251" t="inlineStr">
-        <is>
-          <t>WESTERN UNION PERU S.A.</t>
-        </is>
-      </c>
       <c r="O251" t="n">
         <v>7000002015</v>
       </c>
@@ -12513,11 +12613,6 @@
       <c r="J263" t="n">
         <v>2401</v>
       </c>
-      <c r="L263" t="inlineStr">
-        <is>
-          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
-        </is>
-      </c>
       <c r="O263" t="n">
         <v>7000002016</v>
       </c>
@@ -12978,11 +13073,6 @@
       <c r="J273" t="n">
         <v>2401</v>
       </c>
-      <c r="L273" t="inlineStr">
-        <is>
-          <t>DIAR INGENIEROS S.A.</t>
-        </is>
-      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -13737,11 +13827,6 @@
       <c r="J289" t="n">
         <v>2401</v>
       </c>
-      <c r="L289" t="inlineStr">
-        <is>
-          <t>EMPRESA DE GENERACION ELECTRICA DE AREQUIPA S.A.</t>
-        </is>
-      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -16729,11 +16814,6 @@
           <t>0000010041</t>
         </is>
       </c>
-      <c r="L361" t="inlineStr">
-        <is>
-          <t>KONDU S.A.C</t>
-        </is>
-      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -16778,11 +16858,6 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
-      <c r="L362" t="inlineStr">
-        <is>
-          <t>FIDEICOMISO ELECTROPERU</t>
-        </is>
-      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -16827,11 +16902,6 @@
           <t>0000010041</t>
         </is>
       </c>
-      <c r="L363" t="inlineStr">
-        <is>
-          <t>KALLPA GENERACION SA</t>
-        </is>
-      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -16871,11 +16941,6 @@
       <c r="J364" t="n">
         <v>2401</v>
       </c>
-      <c r="L364" t="inlineStr">
-        <is>
-          <t>ENTIDAD PRESTADORA DE SERVICIOS DE SANEA</t>
-        </is>
-      </c>
       <c r="O364" t="n">
         <v>7000001902</v>
       </c>
@@ -16960,11 +17025,6 @@
       <c r="J366" t="n">
         <v>2401</v>
       </c>
-      <c r="L366" t="inlineStr">
-        <is>
-          <t>COFIDE FID FISE</t>
-        </is>
-      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -17202,11 +17262,6 @@
           <t>0000010041</t>
         </is>
       </c>
-      <c r="L371" t="inlineStr">
-        <is>
-          <t>ORAZUL ENERGY PERU SA</t>
-        </is>
-      </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -17355,11 +17410,6 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
-      <c r="L374" t="inlineStr">
-        <is>
-          <t>WESTERN UNION PERU S.A.</t>
-        </is>
-      </c>
       <c r="O374" t="n">
         <v>7000002001</v>
       </c>
@@ -17919,11 +17969,6 @@
       <c r="J386" t="n">
         <v>2401</v>
       </c>
-      <c r="L386" t="inlineStr">
-        <is>
-          <t>ENTIDAD PRESTADORA DE SERVICIOS DE SANEA</t>
-        </is>
-      </c>
       <c r="O386" t="n">
         <v>7000002066</v>
       </c>
@@ -17966,11 +18011,6 @@
       <c r="J387" t="n">
         <v>2401</v>
       </c>
-      <c r="L387" t="inlineStr">
-        <is>
-          <t>ENTIDAD PRESTADORA DE SERVICIOS DE SANEA</t>
-        </is>
-      </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -19070,11 +19110,6 @@
       <c r="J410" t="n">
         <v>2401</v>
       </c>
-      <c r="L410" t="inlineStr">
-        <is>
-          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
-        </is>
-      </c>
       <c r="O410" t="n">
         <v>7000001996</v>
       </c>
@@ -19122,6 +19157,11 @@
           <t>MUNI DIST INCAHUASI PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q411" t="inlineStr">
+        <is>
+          <t>mpurihuaman@muniincahuasi.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -19161,11 +19201,6 @@
       <c r="J412" t="n">
         <v>2401</v>
       </c>
-      <c r="L412" t="inlineStr">
-        <is>
-          <t>ENTIDAD PRESTADORA DE SERVICIOS DE SANEA</t>
-        </is>
-      </c>
       <c r="O412" t="n">
         <v>7000002067</v>
       </c>
@@ -22308,6 +22343,11 @@
           <t>MUNI DIST POMALCA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q478" t="inlineStr">
+        <is>
+          <t>genarocpc@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
@@ -22352,6 +22392,11 @@
           <t>MUNI DIST POMALCA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q479" t="inlineStr">
+        <is>
+          <t>genarocpc@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -22396,6 +22441,11 @@
           <t>MUNI DIST POMALCA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q480" t="inlineStr">
+        <is>
+          <t>genarocpc@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
@@ -22440,6 +22490,11 @@
           <t>MUNI DIST POMALCA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q481" t="inlineStr">
+        <is>
+          <t>genarocpc@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
@@ -22484,6 +22539,11 @@
           <t>MUNI DIST POMALCA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q482" t="inlineStr">
+        <is>
+          <t>genarocpc@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
@@ -22958,6 +23018,11 @@
           <t>MUNI DIST POMALCA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q492" t="inlineStr">
+        <is>
+          <t>genarocpc@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
@@ -24087,11 +24152,6 @@
           <t>Ref 20103117560-01-F06</t>
         </is>
       </c>
-      <c r="L516" t="inlineStr">
-        <is>
-          <t>VARI ENERGIA SAC</t>
-        </is>
-      </c>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
@@ -25306,11 +25366,6 @@
           <t>S017603022026</t>
         </is>
       </c>
-      <c r="L545" t="inlineStr">
-        <is>
-          <t>LUZ DEL SUR S.A.A.</t>
-        </is>
-      </c>
     </row>
     <row r="546">
       <c r="A546" t="inlineStr">
@@ -25548,11 +25603,6 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
-      <c r="L550" t="inlineStr">
-        <is>
-          <t>WESTERN UNION PERU S.A.</t>
-        </is>
-      </c>
       <c r="O550" t="n">
         <v>7000001737</v>
       </c>
@@ -26112,11 +26162,6 @@
       <c r="J562" t="n">
         <v>2401</v>
       </c>
-      <c r="L562" t="inlineStr">
-        <is>
-          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
-        </is>
-      </c>
       <c r="O562" t="n">
         <v>7000001735</v>
       </c>
@@ -26322,11 +26367,6 @@
       <c r="J566" t="n">
         <v>2401</v>
       </c>
-      <c r="L566" t="inlineStr">
-        <is>
-          <t>VIETTEL PERU S.A.C - CAJ</t>
-        </is>
-      </c>
       <c r="O566" t="n">
         <v>7000002106</v>
       </c>
@@ -26525,11 +26565,6 @@
       <c r="J570" t="n">
         <v>2401</v>
       </c>
-      <c r="L570" t="inlineStr">
-        <is>
-          <t>VIETTEL PERU S.A.C - CAJ</t>
-        </is>
-      </c>
       <c r="O570" t="n">
         <v>7000002105</v>
       </c>
@@ -26769,11 +26804,6 @@
       <c r="J575" t="n">
         <v>2401</v>
       </c>
-      <c r="L575" t="inlineStr">
-        <is>
-          <t>TERMOSELVA S.R.L.</t>
-        </is>
-      </c>
     </row>
     <row r="576">
       <c r="A576" t="inlineStr">
@@ -26818,11 +26848,6 @@
           <t>S018104022026</t>
         </is>
       </c>
-      <c r="L576" t="inlineStr">
-        <is>
-          <t>INLAND ENERGY SAC</t>
-        </is>
-      </c>
     </row>
     <row r="577">
       <c r="A577" t="inlineStr">
@@ -26867,11 +26892,6 @@
           <t>01-F061-00020521</t>
         </is>
       </c>
-      <c r="L577" t="inlineStr">
-        <is>
-          <t>INVERSIONES SHAQSHA S.A.C.</t>
-        </is>
-      </c>
     </row>
     <row r="578">
       <c r="A578" t="inlineStr">
@@ -27966,11 +27986,6 @@
           <t>01-F061-00020467</t>
         </is>
       </c>
-      <c r="L603" t="inlineStr">
-        <is>
-          <t>STATKRAFT PERU SA</t>
-        </is>
-      </c>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
@@ -28114,6 +28129,11 @@
           <t>MUNI DIST MANUEL A MESONES MURO PPT</t>
         </is>
       </c>
+      <c r="Q606" t="inlineStr">
+        <is>
+          <t>seanjuch72@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="607">
       <c r="A607" t="inlineStr">
@@ -28200,11 +28220,6 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
-      <c r="L608" t="inlineStr">
-        <is>
-          <t>WESTERN UNION PERU S.A.</t>
-        </is>
-      </c>
       <c r="O608" t="n">
         <v>7000001608</v>
       </c>
@@ -28252,6 +28267,11 @@
           <t>MUNI DIST MANUEL A MESONES MURO PPT</t>
         </is>
       </c>
+      <c r="Q609" t="inlineStr">
+        <is>
+          <t>seanjuch72@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="610">
       <c r="A610" t="inlineStr">
@@ -28296,11 +28316,6 @@
           <t>Pago beneficiario</t>
         </is>
       </c>
-      <c r="L610" t="inlineStr">
-        <is>
-          <t>ELECTRO DUNAS S.A.A.</t>
-        </is>
-      </c>
     </row>
     <row r="611">
       <c r="A611" t="inlineStr">
@@ -28345,6 +28360,11 @@
           <t>MUNI DIST MANUEL A MESONES MURO PPT</t>
         </is>
       </c>
+      <c r="Q611" t="inlineStr">
+        <is>
+          <t>seanjuch72@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
@@ -28649,6 +28669,11 @@
           <t>MUNI DIST MANUEL A MESONES MURO PPT</t>
         </is>
       </c>
+      <c r="Q617" t="inlineStr">
+        <is>
+          <t>seanjuch72@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="618">
       <c r="A618" t="inlineStr">
@@ -28735,6 +28760,11 @@
           <t>MUNI DIST MANUEL A MESONES MURO PPT</t>
         </is>
       </c>
+      <c r="Q619" t="inlineStr">
+        <is>
+          <t>seanjuch72@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
@@ -28878,11 +28908,6 @@
       <c r="J622" t="n">
         <v>2401</v>
       </c>
-      <c r="L622" t="inlineStr">
-        <is>
-          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
-        </is>
-      </c>
       <c r="O622" t="n">
         <v>7000001606</v>
       </c>
@@ -29585,11 +29610,6 @@
           <t>Pago Fact.20494</t>
         </is>
       </c>
-      <c r="L636" t="inlineStr">
-        <is>
-          <t>TERMOCHILCA S.A.C.</t>
-        </is>
-      </c>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr">
@@ -29634,6 +29654,11 @@
           <t>GR CAJAMARCA-EDUCAC UGEL CELENDIN</t>
         </is>
       </c>
+      <c r="Q637" t="inlineStr">
+        <is>
+          <t>abastecimientos@ugelcelendin.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="638">
       <c r="A638" t="inlineStr">
@@ -29678,11 +29703,6 @@
           <t>Pago Fact.20485</t>
         </is>
       </c>
-      <c r="L638" t="inlineStr">
-        <is>
-          <t>COMPANIA ELECTRICA EL PLATANAL S.A.</t>
-        </is>
-      </c>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr">
@@ -29727,11 +29747,6 @@
           <t>Pago Fact.20505</t>
         </is>
       </c>
-      <c r="L639" t="inlineStr">
-        <is>
-          <t>CELEPSA RENOVABLES SRL</t>
-        </is>
-      </c>
     </row>
     <row r="640">
       <c r="A640" t="inlineStr">
@@ -30734,11 +30749,6 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
-      <c r="L662" t="inlineStr">
-        <is>
-          <t>WESTERN UNION PERU S.A.</t>
-        </is>
-      </c>
       <c r="O662" t="n">
         <v>6900000034</v>
       </c>
@@ -31192,6 +31202,11 @@
           <t>MTC ADMINISTRACION GRAL PPTO 2003</t>
         </is>
       </c>
+      <c r="Q671" t="inlineStr">
+        <is>
+          <t>apaicog@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="672">
       <c r="A672" t="inlineStr">
@@ -31231,11 +31246,6 @@
       <c r="J672" t="n">
         <v>2401</v>
       </c>
-      <c r="L672" t="inlineStr">
-        <is>
-          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
-        </is>
-      </c>
       <c r="O672" t="n">
         <v>6900000023</v>
       </c>
@@ -33205,11 +33215,6 @@
           <t>Pago0002300998-2026-FE</t>
         </is>
       </c>
-      <c r="L713" t="inlineStr">
-        <is>
-          <t>FENIX POWER PERU S.A.</t>
-        </is>
-      </c>
     </row>
     <row r="714">
       <c r="A714" t="inlineStr">
@@ -33254,6 +33259,11 @@
           <t>SERNANP SEDE LAMBAYEQUE ENCARGOS</t>
         </is>
       </c>
+      <c r="Q714" t="inlineStr">
+        <is>
+          <t>lvalles@sernanp.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="715">
       <c r="A715" t="inlineStr">
@@ -33441,11 +33451,6 @@
       <c r="J718" t="n">
         <v>2401</v>
       </c>
-      <c r="L718" t="inlineStr">
-        <is>
-          <t>EMPRESA DE GENERACION ELECTRICA SAN GABAN S.A.</t>
-        </is>
-      </c>
     </row>
     <row r="719">
       <c r="A719" t="inlineStr">
@@ -34432,11 +34437,6 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
-      <c r="L741" t="inlineStr">
-        <is>
-          <t>WESTERN UNION PERU S.A.</t>
-        </is>
-      </c>
     </row>
     <row r="742">
       <c r="A742" t="inlineStr">
@@ -34617,6 +34617,11 @@
           <t>MUNI PROV CHICLAYO PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q745" t="inlineStr">
+        <is>
+          <t>logistica@munichiclayo.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="746">
       <c r="A746" t="inlineStr">
@@ -35620,6 +35625,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q766" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="767">
       <c r="A767" t="inlineStr">
@@ -35664,6 +35674,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q767" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="768">
       <c r="A768" t="inlineStr">
@@ -35948,6 +35963,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q773" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="774">
       <c r="A774" t="inlineStr">
@@ -36081,11 +36101,6 @@
       <c r="J776" t="n">
         <v>2401</v>
       </c>
-      <c r="L776" t="inlineStr">
-        <is>
-          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
-        </is>
-      </c>
     </row>
     <row r="777">
       <c r="A777" t="inlineStr">
@@ -36640,6 +36655,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q787" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="788">
       <c r="A788" t="inlineStr">
@@ -36877,6 +36897,11 @@
           <t>PROGRAMA NACIONAL DE EMPLEO JUVENIL</t>
         </is>
       </c>
+      <c r="Q792" t="inlineStr">
+        <is>
+          <t>aabrilr@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="793">
       <c r="A793" t="inlineStr">
@@ -36968,6 +36993,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q794" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="795">
       <c r="A795" t="inlineStr">
@@ -37012,11 +37042,6 @@
           <t>PAGO DE PROVEEDORES</t>
         </is>
       </c>
-      <c r="L795" t="inlineStr">
-        <is>
-          <t>FIDEICOMISO ELECTROPERU</t>
-        </is>
-      </c>
     </row>
     <row r="796">
       <c r="A796" t="inlineStr">
@@ -37061,6 +37086,11 @@
           <t>PROGRAMA NACIONAL DE EMPLEO JUVENIL</t>
         </is>
       </c>
+      <c r="Q796" t="inlineStr">
+        <is>
+          <t>aabrilr@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="797">
       <c r="A797" t="inlineStr">
@@ -37157,6 +37187,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q798" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="799">
       <c r="A799" t="inlineStr">
@@ -37250,6 +37285,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q800" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="801">
       <c r="A801" t="inlineStr">
@@ -37382,11 +37422,6 @@
       <c r="J803" t="n">
         <v>2401</v>
       </c>
-      <c r="L803" t="inlineStr">
-        <is>
-          <t>HYDRO GLOBAL PERU S.A.C.</t>
-        </is>
-      </c>
     </row>
     <row r="804">
       <c r="A804" t="inlineStr">
@@ -37429,11 +37464,6 @@
       <c r="K804" t="inlineStr">
         <is>
           <t>Pago beneficiario</t>
-        </is>
-      </c>
-      <c r="L804" t="inlineStr">
-        <is>
-          <t>SINDICATO ENERGETICO S.A.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync project from Banco1 into current workspace
</commit_message>
<xml_diff>
--- a/files/asientos.xlsx
+++ b/files/asientos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P805"/>
+  <dimension ref="A1:Q805"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -517,6 +517,11 @@
           <t>Correos</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1284,6 +1289,11 @@
           <t>UNIV NAC PEDRO RUIZ GALLO PTO 2003</t>
         </is>
       </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>minonanve@unprg.edu.pe</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1328,6 +1338,11 @@
           <t>UNIV NAC PEDRO RUIZ GALLO PTO 2003</t>
         </is>
       </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>minonanve@unprg.edu.pe</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1830,6 +1845,11 @@
           <t>MUNI DIST MOCHUMI PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>u212prac01@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2006,6 +2026,11 @@
           <t>MUNI DIST ANGUIA</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>ronaldlabans@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2050,6 +2075,11 @@
           <t>REGION CAJAMARCA-CHOTA PPTO</t>
         </is>
       </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>carlosbva8@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2479,6 +2509,11 @@
           <t>MUNI DIST LAJAS</t>
         </is>
       </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>tesoreria@munilajas.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2523,6 +2558,11 @@
           <t>MUNI DIST ANGUIA</t>
         </is>
       </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>ronaldlabans@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2567,6 +2607,11 @@
           <t>MUNI DIST ANGUIA</t>
         </is>
       </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>ronaldlabans@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2701,7 +2746,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>TRABAJADOR-72714263</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -2802,6 +2847,11 @@
           <t>DIREC AVIACION POLICIAL PTO 2003</t>
         </is>
       </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>depsam.lambayeque@policia.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2848,7 +2898,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16733606</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2947,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>TRABAJADOR-40554960</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -2946,7 +2996,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16736597</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -2993,6 +3043,11 @@
           <t>SUPERINT NAC FISCALIZACION LABORAL-</t>
         </is>
       </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>lruizr@sunafil.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3093,7 +3148,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17450838</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3189,6 +3244,11 @@
           <t>MUNI DIST ANGUIA</t>
         </is>
       </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>ronaldlabans@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3235,7 +3295,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16637191</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3282,6 +3342,11 @@
           <t>ORG SUP INVERSION ENERGIA Y MINERIA</t>
         </is>
       </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>ycruzado@osinergmin.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3328,7 +3393,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16562947</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3442,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17450805</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3426,7 +3491,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17624824</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3475,7 +3540,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16689857</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3524,7 +3589,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16796766</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3612,7 +3677,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16761556</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -4778,6 +4843,11 @@
           <t>IPD PPTO 2003</t>
         </is>
       </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>malvites@ipd.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4866,6 +4936,11 @@
           <t>MUNI DIST PITIPO PPTO</t>
         </is>
       </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>jvaleriano1112@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4996,6 +5071,11 @@
           <t>CENTRO DE FORMACION EN TURISMO</t>
         </is>
       </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>dllaguento@cenfotur.edu.pe</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5040,6 +5120,11 @@
           <t>REGION LAMBAYEQUE-AGRICULTURA PPTO</t>
         </is>
       </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>graservicios2024@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5505,7 +5590,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16761208</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O111" t="n">
@@ -5599,6 +5684,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5845,6 +5935,11 @@
           <t>REGION LAMBAYEQUE-AGRICULTURA PPTO</t>
         </is>
       </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>graservicios2024@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -5889,6 +5984,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -5935,7 +6035,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17625165</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O120" t="n">
@@ -6071,6 +6171,11 @@
           <t>MUNI DIST MIRACOSTA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>gorderiquev@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6115,6 +6220,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -6161,7 +6271,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16759780</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O125" t="n">
@@ -6211,6 +6321,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6314,7 +6429,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>TRABAJADOR-43157511</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -6361,6 +6476,11 @@
           <t>MUNI DIST MIRACOSTA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>gorderiquev@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6452,6 +6572,11 @@
           <t>MUNI DIST MIRACOSTA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>gorderiquev@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6496,6 +6621,11 @@
           <t>MTC ADMINISTRACION GRAL PPTO 2003</t>
         </is>
       </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>apaicog@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6542,7 +6672,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>TRABAJADOR-26737638</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O133" t="n">
@@ -6594,7 +6724,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>TRABAJADOR-40179551</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O134" t="n">
@@ -6646,7 +6776,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>TRABAJADOR-45385378</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O135" t="n">
@@ -6740,6 +6870,11 @@
           <t>MUNI DIST MIRACOSTA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>gorderiquev@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6784,6 +6919,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6828,6 +6968,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -6872,6 +7017,11 @@
           <t>GR CAJAMARCA-EDUCAC UGEL CELENDIN</t>
         </is>
       </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>abastecimientos@ugelcelendin.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6916,6 +7066,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -6960,6 +7115,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -7004,6 +7164,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -7048,6 +7213,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -7149,6 +7319,11 @@
           <t>MUNI DIST MIRACOSTA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>gorderiquev@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -7193,6 +7368,11 @@
           <t>MUNI DIST MIRACOSTA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>gorderiquev@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -7237,6 +7417,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -7281,6 +7466,11 @@
           <t>MUNI DIST CHONGOYAPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>mdch.abastecimiento.2019@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -8526,6 +8716,11 @@
           <t>REGION CAJAMARCA-SALUD CUTERVO</t>
         </is>
       </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>fsoberon05@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -9093,7 +9288,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>TRABAJADOR-40042745</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O189" t="n">
@@ -9585,7 +9780,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16729500</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O199" t="n">
@@ -9832,7 +10027,7 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16753094</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O204" t="n">
@@ -9988,7 +10183,7 @@
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>TRABAJADOR-43157511</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O207" t="n">
@@ -10223,7 +10418,7 @@
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16683457</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O212" t="n">
@@ -10745,7 +10940,7 @@
       </c>
       <c r="M223" t="inlineStr">
         <is>
-          <t>TRABAJADOR-41756285</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O223" t="n">
@@ -13029,7 +13224,7 @@
       </c>
       <c r="M274" t="inlineStr">
         <is>
-          <t>TRABAJADOR-7531871</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O274" t="n">
@@ -13257,7 +13452,7 @@
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16754694</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -13464,7 +13659,7 @@
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16735252</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O283" t="n">
@@ -13516,7 +13711,7 @@
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16423762</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O284" t="n">
@@ -13788,7 +13983,7 @@
       </c>
       <c r="M290" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16762908</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -18247,7 +18442,7 @@
       </c>
       <c r="M393" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16661452</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -18296,7 +18491,7 @@
       </c>
       <c r="M394" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16715161</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -19025,7 +19220,7 @@
       </c>
       <c r="M409" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16753094</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O409" t="n">
@@ -19122,6 +19317,11 @@
           <t>MUNI DIST INCAHUASI PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q411" t="inlineStr">
+        <is>
+          <t>mpurihuaman@muniincahuasi.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -19386,7 +19586,7 @@
       </c>
       <c r="M416" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16659349</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O416" t="n">
@@ -19438,7 +19638,7 @@
       </c>
       <c r="M417" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17631880</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O417" t="n">
@@ -22308,6 +22508,11 @@
           <t>MUNI DIST POMALCA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q478" t="inlineStr">
+        <is>
+          <t>genarocpc@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
@@ -22352,6 +22557,11 @@
           <t>MUNI DIST POMALCA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q479" t="inlineStr">
+        <is>
+          <t>genarocpc@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -22396,6 +22606,11 @@
           <t>MUNI DIST POMALCA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q480" t="inlineStr">
+        <is>
+          <t>genarocpc@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
@@ -22440,6 +22655,11 @@
           <t>MUNI DIST POMALCA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q481" t="inlineStr">
+        <is>
+          <t>genarocpc@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
@@ -22484,6 +22704,11 @@
           <t>MUNI DIST POMALCA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q482" t="inlineStr">
+        <is>
+          <t>genarocpc@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
@@ -22530,7 +22755,7 @@
       </c>
       <c r="M483" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17624824</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O483" t="n">
@@ -22676,7 +22901,7 @@
       </c>
       <c r="M486" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17617984</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O486" t="n">
@@ -22728,7 +22953,7 @@
       </c>
       <c r="M487" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16715161</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O487" t="n">
@@ -22958,6 +23183,11 @@
           <t>MUNI DIST POMALCA PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q492" t="inlineStr">
+        <is>
+          <t>genarocpc@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
@@ -23991,7 +24221,7 @@
       </c>
       <c r="M514" t="inlineStr">
         <is>
-          <t>TRABAJADOR-40179551</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -24040,7 +24270,7 @@
       </c>
       <c r="M515" t="inlineStr">
         <is>
-          <t>TRABAJADOR-40179551</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -26223,7 +26453,7 @@
       </c>
       <c r="M564" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16754694</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -26680,7 +26910,7 @@
       </c>
       <c r="M573" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16687406</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O573" t="n">
@@ -28114,6 +28344,11 @@
           <t>MUNI DIST MANUEL A MESONES MURO PPT</t>
         </is>
       </c>
+      <c r="Q606" t="inlineStr">
+        <is>
+          <t>seanjuch72@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="607">
       <c r="A607" t="inlineStr">
@@ -28252,6 +28487,11 @@
           <t>MUNI DIST MANUEL A MESONES MURO PPT</t>
         </is>
       </c>
+      <c r="Q609" t="inlineStr">
+        <is>
+          <t>seanjuch72@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="610">
       <c r="A610" t="inlineStr">
@@ -28345,6 +28585,11 @@
           <t>MUNI DIST MANUEL A MESONES MURO PPT</t>
         </is>
       </c>
+      <c r="Q611" t="inlineStr">
+        <is>
+          <t>seanjuch72@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
@@ -28649,6 +28894,11 @@
           <t>MUNI DIST MANUEL A MESONES MURO PPT</t>
         </is>
       </c>
+      <c r="Q617" t="inlineStr">
+        <is>
+          <t>seanjuch72@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="618">
       <c r="A618" t="inlineStr">
@@ -28735,6 +28985,11 @@
           <t>MUNI DIST MANUEL A MESONES MURO PPT</t>
         </is>
       </c>
+      <c r="Q619" t="inlineStr">
+        <is>
+          <t>seanjuch72@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
@@ -29229,7 +29484,7 @@
       </c>
       <c r="M629" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16683457</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O629" t="n">
@@ -29489,7 +29744,7 @@
       </c>
       <c r="M634" t="inlineStr">
         <is>
-          <t>TRABAJADOR-45080863</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -29538,7 +29793,7 @@
       </c>
       <c r="M635" t="inlineStr">
         <is>
-          <t>TRABAJADOR-72644789</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -29634,6 +29889,11 @@
           <t>GR CAJAMARCA-EDUCAC UGEL CELENDIN</t>
         </is>
       </c>
+      <c r="Q637" t="inlineStr">
+        <is>
+          <t>abastecimientos@ugelcelendin.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="638">
       <c r="A638" t="inlineStr">
@@ -31192,6 +31452,11 @@
           <t>MTC ADMINISTRACION GRAL PPTO 2003</t>
         </is>
       </c>
+      <c r="Q671" t="inlineStr">
+        <is>
+          <t>apaicog@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="672">
       <c r="A672" t="inlineStr">
@@ -31475,7 +31740,7 @@
       </c>
       <c r="M677" t="inlineStr">
         <is>
-          <t>TRABAJADOR-43157511</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O677" t="n">
@@ -31906,7 +32171,7 @@
       </c>
       <c r="M686" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16733606</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O686" t="n">
@@ -32005,7 +32270,7 @@
       </c>
       <c r="M688" t="inlineStr">
         <is>
-          <t>TRABAJADOR-41652040</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O688" t="n">
@@ -32443,7 +32708,7 @@
       </c>
       <c r="M697" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16702986</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O697" t="n">
@@ -32495,7 +32760,7 @@
       </c>
       <c r="M698" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16590196</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -33155,7 +33420,7 @@
       </c>
       <c r="M712" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16722058</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O712" t="n">
@@ -33254,6 +33519,11 @@
           <t>SERNANP SEDE LAMBAYEQUE ENCARGOS</t>
         </is>
       </c>
+      <c r="Q714" t="inlineStr">
+        <is>
+          <t>lvalles@sernanp.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="715">
       <c r="A715" t="inlineStr">
@@ -33347,7 +33617,7 @@
       </c>
       <c r="M716" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16423762</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -33396,7 +33666,7 @@
       </c>
       <c r="M717" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16722058</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O717" t="n">
@@ -34617,6 +34887,11 @@
           <t>MUNI PROV CHICLAYO PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q745" t="inlineStr">
+        <is>
+          <t>logistica@munichiclayo.gob.pe</t>
+        </is>
+      </c>
     </row>
     <row r="746">
       <c r="A746" t="inlineStr">
@@ -35427,7 +35702,7 @@
       </c>
       <c r="M762" t="inlineStr">
         <is>
-          <t>TRABAJADOR-42853214</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -35620,6 +35895,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q766" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="767">
       <c r="A767" t="inlineStr">
@@ -35664,6 +35944,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q767" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="768">
       <c r="A768" t="inlineStr">
@@ -35948,6 +36233,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q773" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="774">
       <c r="A774" t="inlineStr">
@@ -36189,7 +36479,7 @@
       </c>
       <c r="M778" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16729500</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O778" t="n">
@@ -36444,7 +36734,7 @@
       </c>
       <c r="M783" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16761556</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O783" t="n">
@@ -36538,7 +36828,7 @@
       </c>
       <c r="M785" t="inlineStr">
         <is>
-          <t>TRABAJADOR-45080863</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O785" t="n">
@@ -36590,7 +36880,7 @@
       </c>
       <c r="M786" t="inlineStr">
         <is>
-          <t>TRABAJADOR-45080863</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O786" t="n">
@@ -36640,6 +36930,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q787" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="788">
       <c r="A788" t="inlineStr">
@@ -36827,7 +37122,7 @@
       </c>
       <c r="M791" t="inlineStr">
         <is>
-          <t>TRABAJADOR-26737638</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O791" t="n">
@@ -36877,6 +37172,11 @@
           <t>PROGRAMA NACIONAL DE EMPLEO JUVENIL</t>
         </is>
       </c>
+      <c r="Q792" t="inlineStr">
+        <is>
+          <t>aabrilr@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="793">
       <c r="A793" t="inlineStr">
@@ -36968,6 +37268,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q794" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="795">
       <c r="A795" t="inlineStr">
@@ -37061,6 +37366,11 @@
           <t>PROGRAMA NACIONAL DE EMPLEO JUVENIL</t>
         </is>
       </c>
+      <c r="Q796" t="inlineStr">
+        <is>
+          <t>aabrilr@distriluz.com.pe</t>
+        </is>
+      </c>
     </row>
     <row r="797">
       <c r="A797" t="inlineStr">
@@ -37107,7 +37417,7 @@
       </c>
       <c r="M797" t="inlineStr">
         <is>
-          <t>TRABAJADOR-3701237</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O797" t="n">
@@ -37157,6 +37467,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q798" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="799">
       <c r="A799" t="inlineStr">
@@ -37203,7 +37518,7 @@
       </c>
       <c r="M799" t="inlineStr">
         <is>
-          <t>TRABAJADOR-44465574</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -37250,6 +37565,11 @@
           <t>MUNI DIST MORROPE PRESUPUESTO</t>
         </is>
       </c>
+      <c r="Q800" t="inlineStr">
+        <is>
+          <t>santamariabancesleydy@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="801">
       <c r="A801" t="inlineStr">
@@ -37340,7 +37660,7 @@
       </c>
       <c r="M802" t="inlineStr">
         <is>
-          <t>TRABAJADOR-71003287</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>

</xml_diff>